<commit_message>
feat: tipo de acompanhante "Familiar"
</commit_message>
<xml_diff>
--- a/public/modelo_participantes.xlsx
+++ b/public/modelo_participantes.xlsx
@@ -27989,7 +27989,7 @@
       <formula1>=Listas!$A$2:$A$3</formula1>
     </dataValidation>
     <dataValidation sqref="I2:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor inválido" error="Escolha um valor da lista." type="list">
-      <formula1>=Listas!$C$2:$C$5</formula1>
+      <formula1>=Listas!$C$2:$C$6</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Valor inválido" error="Escolha um valor da lista." type="list">
       <formula1>=Listas!$D$2:$D$3</formula1>
@@ -28114,7 +28114,7 @@
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>Professor parceiro</t>
+          <t>Familiar</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
@@ -28136,7 +28136,7 @@
     <row r="4">
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Colaborador</t>
+          <t>Professor parceiro</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
@@ -28148,7 +28148,7 @@
     <row r="5">
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Amigo</t>
+          <t>Colaborador</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -28158,6 +28158,11 @@
       </c>
     </row>
     <row r="6">
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Amigo</t>
+        </is>
+      </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
           <t>5º ciclo</t>

</xml_diff>